<commit_message>
chore: actualizar plan de construccion
</commit_message>
<xml_diff>
--- a/Plan_cosntruccion.xlsx
+++ b/Plan_cosntruccion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Rov\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F635B4E-163B-43B3-9DC2-F7D1C4E64C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F3984F2-D669-43A9-B99E-D4786F0BE957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{75C40051-293E-4382-8A6D-0D6B95F2BCBB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{75C40051-293E-4382-8A6D-0D6B95F2BCBB}"/>
   </bookViews>
   <sheets>
     <sheet name="Tablero" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="365">
   <si>
     <t>Cronograma — Montaje ROV Nivel B (ArduSub / ArduPilot)</t>
   </si>
@@ -898,9 +898,6 @@
     <t>BOM — Lista de materiales ROV Nivel B (equivalente FIFISH V6)</t>
   </si>
   <si>
-    <t>Build ArduSub clase BlueROV2 (6 thrusters vectored). Costos en USD = ESTIMADOS de planificación, a confirmar contra bom-final-nivel-b.md y matriz-proveedores-rov.md. Azul = dato a editar.</t>
-  </si>
-  <si>
     <t>Categoría</t>
   </si>
   <si>
@@ -913,24 +910,247 @@
     <t>Costo unit. est. (USD)</t>
   </si>
   <si>
-    <t>Costo línea</t>
-  </si>
-  <si>
     <t>Fuente sugerida</t>
   </si>
   <si>
     <t>Notas / lección del V6</t>
+  </si>
+  <si>
+    <t>Build ArduSub clase BlueROV2 (6 thrusters, frame vectorizado). Costos USD = ESTIMADOS de planificación, a confirmar contra bom-final-nivel-b.md y matriz-proveedores-rov.md. Texto azul = dato editable.</t>
+  </si>
+  <si>
+    <t>Costo línea (USD)</t>
+  </si>
+  <si>
+    <t>Control y cómputo</t>
+  </si>
+  <si>
+    <t>Raspberry Pi 4 (4 GB) — companion BlueOS</t>
+  </si>
+  <si>
+    <t>Navigator Flight Controller (Blue Robotics)</t>
+  </si>
+  <si>
+    <t>microSD 32 GB (imagen BlueOS)</t>
+  </si>
+  <si>
+    <t>Disipador + ventilación interna</t>
+  </si>
+  <si>
+    <t>Thruster T200 (3 CW + 3 CCW)</t>
+  </si>
+  <si>
+    <t>ESC Basic 30A (BLHeli)</t>
+  </si>
+  <si>
+    <t>Energía</t>
+  </si>
+  <si>
+    <t>Batería Li-ion 4S ~18 Ah (14,8 V)</t>
+  </si>
+  <si>
+    <t>Cargador balanceador 4S</t>
+  </si>
+  <si>
+    <t>Power Sense Module (PSM)</t>
+  </si>
+  <si>
+    <t>UBEC 5 V / 6 A</t>
+  </si>
+  <si>
+    <t>Fusible principal + portafusible</t>
+  </si>
+  <si>
+    <t>Cable estañado (tinned) surtido</t>
+  </si>
+  <si>
+    <t>Bar30 profundidad/temp (I2C)</t>
+  </si>
+  <si>
+    <t>Sonda de fuga (leak sensor SOS)</t>
+  </si>
+  <si>
+    <t>Comunicación</t>
+  </si>
+  <si>
+    <t>Fathom-X Tether Interface (par)</t>
+  </si>
+  <si>
+    <t>Tether 100 m neutralmente flotante</t>
+  </si>
+  <si>
+    <t>Adaptador USB–Ethernet</t>
+  </si>
+  <si>
+    <t>Cable Ethernet + JST-GH surtido</t>
+  </si>
+  <si>
+    <t>Visión</t>
+  </si>
+  <si>
+    <t>Cámara low-light USB/IP</t>
+  </si>
+  <si>
+    <t>Luces LED sumergibles (par)</t>
+  </si>
+  <si>
+    <t>Casco/enclosure + tapas (4")</t>
+  </si>
+  <si>
+    <t>Penetradores surtidos</t>
+  </si>
+  <si>
+    <t>O-rings + grasa de silicona</t>
+  </si>
+  <si>
+    <t>Frame / estructura</t>
+  </si>
+  <si>
+    <t>Flotación (foam) + lastre</t>
+  </si>
+  <si>
+    <t>Control operador</t>
+  </si>
+  <si>
+    <t>Joystick USB (gamepad)</t>
+  </si>
+  <si>
+    <t>Consumibles</t>
+  </si>
+  <si>
+    <t>Kit de rescate + consumibles pileta</t>
+  </si>
+  <si>
+    <t>AliExpress / oficial</t>
+  </si>
+  <si>
+    <t>Cerebro de alto nivel; alejarla de la zona húmeda y darle disipación.</t>
+  </si>
+  <si>
+    <t>Blue Robotics (oficial)</t>
+  </si>
+  <si>
+    <t>Reemplaza el autopiloto propietario del V6; firmware abierto = reparable.</t>
+  </si>
+  <si>
+    <t>Local / AliExpress</t>
+  </si>
+  <si>
+    <t>Tener 2 clonadas: una SD que falla deja el ROV mudo.</t>
+  </si>
+  <si>
+    <t>AliExpress</t>
+  </si>
+  <si>
+    <t>El V6 calentó 40–45 °C; gestionar térmica desde el diseño.</t>
+  </si>
+  <si>
+    <t>La falla del V6 fue 1 thruster: montarlos accesibles y con conector estanco individual.</t>
+  </si>
+  <si>
+    <t>Blue Robotics / AliExpress</t>
+  </si>
+  <si>
+    <t>1 ESC por motor; canal dañado = falla de fase. Dejar 1 de repuesto.</t>
+  </si>
+  <si>
+    <t>Local certificada</t>
+  </si>
+  <si>
+    <t>Li-ion + agua salada = riesgo térmico; comprar recién con cargador/BMS confirmados.</t>
+  </si>
+  <si>
+    <t>Local / oficial</t>
+  </si>
+  <si>
+    <t>No comprar batería sin este confirmado (regla de seguridad del schedule).</t>
+  </si>
+  <si>
+    <t>Blue Robotics</t>
+  </si>
+  <si>
+    <t>Monitoreo V/A para failsafe de batería baja.</t>
+  </si>
+  <si>
+    <t>Alimentación limpia a Pi/Navigator, separada de la potencia de motores.</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Protección ante corto por corrosión o ingreso de agua.</t>
+  </si>
+  <si>
+    <t>Blue Robotics / local</t>
+  </si>
+  <si>
+    <t>Cobre estañado resiste la corrosión salina mejor que el cobre desnudo.</t>
+  </si>
+  <si>
+    <t>Habilita depth hold; también vigila temperatura interna.</t>
+  </si>
+  <si>
+    <t>Lo que le faltó al V6: alarma temprana antes del daño mayor.</t>
+  </si>
+  <si>
+    <t>Video + MAVLink por un par; probar temprano con tramo corto (riesgo del schedule).</t>
+  </si>
+  <si>
+    <t>Largo lead time: pedir en la semana 1.</t>
+  </si>
+  <si>
+    <t>Enlace directo laptop ↔ BlueOS (red 192.168.2.x).</t>
+  </si>
+  <si>
+    <t>Señal separada de potencia; alivio de tracción en cada conector.</t>
+  </si>
+  <si>
+    <t>La condensación en el domo fue síntoma clave del V6: sellar bien la óptica.</t>
+  </si>
+  <si>
+    <t>Opcional pero recomendado para pileta y aguas turbias.</t>
+  </si>
+  <si>
+    <t>No abrir cascos sellados sin re-test; diseñar apertura mantenible.</t>
+  </si>
+  <si>
+    <t>Punto típico de fuga; usar el correcto por diámetro de cable.</t>
+  </si>
+  <si>
+    <t>Solo grasa de silicona (nunca base petróleo); un pelo o sal = fuga.</t>
+  </si>
+  <si>
+    <t>AliExpress / impresión 3D</t>
+  </si>
+  <si>
+    <t>Layout que separe potencia y señal, con thrusters accesibles.</t>
+  </si>
+  <si>
+    <t>Ajuste de trim neutro o levemente positivo.</t>
+  </si>
+  <si>
+    <t>Interfaz de pilotaje en QGC/Cockpit.</t>
+  </si>
+  <si>
+    <t>Cuerda de recuperación y repuestos para las sesiones de validación.</t>
+  </si>
+  <si>
+    <t>TOTAL ESTIMADO (USD)</t>
+  </si>
+  <si>
+    <t>Presupuesto est. (BOM)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;S&quot;0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1035,6 +1255,44 @@
       <b/>
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F3864"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F3864"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1591,7 +1849,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1659,8 +1917,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1825,6 +2081,89 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2355,7 +2694,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="426" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="557" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -2389,356 +2728,365 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="68" t="s">
         <v>240</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="32" t="s">
         <v>241</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="91" t="s">
+      <c r="A4" s="89" t="s">
         <v>242</v>
       </c>
-      <c r="B4" s="91"/>
-      <c r="D4" s="91" t="s">
+      <c r="B4" s="89"/>
+      <c r="D4" s="89" t="s">
         <v>249</v>
       </c>
-      <c r="E4" s="91"/>
+      <c r="E4" s="89"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="93" t="s">
+      <c r="A5" s="91" t="s">
         <v>243</v>
       </c>
-      <c r="B5" s="71">
+      <c r="B5" s="69">
         <f>COUNTA(Cronograma!A5:A37)</f>
         <v>33</v>
       </c>
-      <c r="D5" s="93" t="s">
+      <c r="D5" s="91" t="s">
         <v>250</v>
       </c>
-      <c r="E5" s="71">
+      <c r="E5" s="69">
         <f>COUNTIF(Gates!D5:D12,"Hecho")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="93" t="s">
+      <c r="A6" s="91" t="s">
         <v>244</v>
       </c>
-      <c r="B6" s="71">
+      <c r="B6" s="69">
         <f>COUNTIF(Cronograma!I5:I37,"Hecho")</f>
         <v>0</v>
       </c>
-      <c r="D6" s="93" t="s">
+      <c r="D6" s="91" t="s">
         <v>251</v>
       </c>
-      <c r="E6" s="71">
+      <c r="E6" s="69">
         <f>COUNTA(Gates!A5:A12)</f>
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="93" t="s">
+      <c r="A7" s="91" t="s">
         <v>245</v>
       </c>
-      <c r="B7" s="71">
+      <c r="B7" s="69">
         <f>COUNTIF(Cronograma!I5:I37,"En curso")</f>
         <v>0</v>
       </c>
-      <c r="D7" s="94" t="s">
+      <c r="D7" s="92" t="s">
         <v>252</v>
       </c>
-      <c r="E7" s="72">
+      <c r="E7" s="70">
         <f>IF(E6=0,0,E5/E6)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="93" t="s">
+      <c r="A8" s="91" t="s">
         <v>246</v>
       </c>
-      <c r="B8" s="71">
+      <c r="B8" s="69">
         <f>COUNTIF(Cronograma!I5:I37,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="71"/>
+      <c r="D8" s="91"/>
+      <c r="E8" s="69"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="93" t="s">
+      <c r="A9" s="91" t="s">
         <v>247</v>
       </c>
-      <c r="B9" s="71">
+      <c r="B9" s="69">
         <f>COUNTIF(Cronograma!I5:I37,"Pendiente")</f>
         <v>33</v>
       </c>
-      <c r="D9" s="95" t="s">
+      <c r="D9" s="93" t="s">
         <v>253</v>
       </c>
-      <c r="E9" s="92"/>
+      <c r="E9" s="90"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="93" t="s">
+      <c r="A10" s="91" t="s">
         <v>248</v>
       </c>
-      <c r="B10" s="72">
+      <c r="B10" s="70">
         <f>IF(B5=0,0,B6/B5)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="93" t="s">
+      <c r="D10" s="91" t="s">
         <v>254</v>
       </c>
-      <c r="E10" s="71">
+      <c r="E10" s="69">
         <f>COUNTIF(Riesgos!C5:C11,"Alto")</f>
         <v>3</v>
       </c>
     </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D11" s="121" t="s">
+        <v>364</v>
+      </c>
+      <c r="E11" s="122">
+        <f>BOM!E32</f>
+        <v>3877</v>
+      </c>
+    </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="91" t="s">
+      <c r="A12" s="89" t="s">
         <v>255</v>
       </c>
-      <c r="B12" s="91"/>
-      <c r="C12" s="91"/>
-      <c r="D12" s="91"/>
-      <c r="E12" s="91"/>
-      <c r="F12" s="91"/>
+      <c r="B12" s="89"/>
+      <c r="C12" s="89"/>
+      <c r="D12" s="89"/>
+      <c r="E12" s="89"/>
+      <c r="F12" s="89"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="74" t="s">
+      <c r="A13" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="75" t="s">
+      <c r="B13" s="73" t="s">
         <v>256</v>
       </c>
-      <c r="C13" s="76" t="s">
+      <c r="C13" s="74" t="s">
         <v>257</v>
       </c>
-      <c r="D13" s="76" t="s">
+      <c r="D13" s="74" t="s">
         <v>258</v>
       </c>
-      <c r="E13" s="76" t="s">
+      <c r="E13" s="74" t="s">
         <v>244</v>
       </c>
-      <c r="F13" s="77" t="s">
+      <c r="F13" s="75" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="83" t="s">
+      <c r="A14" s="81" t="s">
         <v>260</v>
       </c>
-      <c r="B14" s="38" t="s">
+      <c r="B14" s="36" t="s">
         <v>261</v>
       </c>
-      <c r="C14" s="78" t="s">
+      <c r="C14" s="76" t="s">
         <v>262</v>
       </c>
-      <c r="D14" s="78">
+      <c r="D14" s="76">
         <f>COUNTIF(Cronograma!$A$5:$A$37,$A14&amp;"*")</f>
         <v>1</v>
       </c>
-      <c r="E14" s="78">
+      <c r="E14" s="76">
         <f>COUNTIFS(Cronograma!$A$5:$A$37,$A14&amp;"*",Cronograma!$I$5:$I$37,"Hecho")</f>
         <v>0</v>
       </c>
-      <c r="F14" s="79">
+      <c r="F14" s="77">
         <f>IF(D14=0,0,E14/D14)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="84" t="s">
+      <c r="A15" s="82" t="s">
         <v>263</v>
       </c>
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="78" t="s">
+      <c r="C15" s="76" t="s">
         <v>264</v>
       </c>
-      <c r="D15" s="78">
+      <c r="D15" s="76">
         <f>COUNTIF(Cronograma!$A$5:$A$37,$A15&amp;"*")</f>
         <v>4</v>
       </c>
-      <c r="E15" s="78">
+      <c r="E15" s="76">
         <f>COUNTIFS(Cronograma!$A$5:$A$37,$A15&amp;"*",Cronograma!$I$5:$I$37,"Hecho")</f>
         <v>0</v>
       </c>
-      <c r="F15" s="79">
+      <c r="F15" s="77">
         <f t="shared" ref="F15:F21" si="0">IF(D15=0,0,E15/D15)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="85" t="s">
+      <c r="A16" s="83" t="s">
         <v>265</v>
       </c>
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="36" t="s">
         <v>266</v>
       </c>
-      <c r="C16" s="78" t="s">
+      <c r="C16" s="76" t="s">
         <v>267</v>
       </c>
-      <c r="D16" s="78">
+      <c r="D16" s="76">
         <f>COUNTIF(Cronograma!$A$5:$A$37,$A16&amp;"*")</f>
         <v>7</v>
       </c>
-      <c r="E16" s="78">
+      <c r="E16" s="76">
         <f>COUNTIFS(Cronograma!$A$5:$A$37,$A16&amp;"*",Cronograma!$I$5:$I$37,"Hecho")</f>
         <v>0</v>
       </c>
-      <c r="F16" s="79">
+      <c r="F16" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="86" t="s">
+      <c r="A17" s="84" t="s">
         <v>268</v>
       </c>
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="36" t="s">
         <v>269</v>
       </c>
-      <c r="C17" s="78" t="s">
+      <c r="C17" s="76" t="s">
         <v>270</v>
       </c>
-      <c r="D17" s="78">
+      <c r="D17" s="76">
         <f>COUNTIF(Cronograma!$A$5:$A$37,$A17&amp;"*")</f>
         <v>5</v>
       </c>
-      <c r="E17" s="78">
+      <c r="E17" s="76">
         <f>COUNTIFS(Cronograma!$A$5:$A$37,$A17&amp;"*",Cronograma!$I$5:$I$37,"Hecho")</f>
         <v>0</v>
       </c>
-      <c r="F17" s="79">
+      <c r="F17" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="87" t="s">
+      <c r="A18" s="85" t="s">
         <v>271</v>
       </c>
-      <c r="B18" s="38" t="s">
+      <c r="B18" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="C18" s="78" t="s">
+      <c r="C18" s="76" t="s">
         <v>272</v>
       </c>
-      <c r="D18" s="78">
+      <c r="D18" s="76">
         <f>COUNTIF(Cronograma!$A$5:$A$37,$A18&amp;"*")</f>
         <v>4</v>
       </c>
-      <c r="E18" s="78">
+      <c r="E18" s="76">
         <f>COUNTIFS(Cronograma!$A$5:$A$37,$A18&amp;"*",Cronograma!$I$5:$I$37,"Hecho")</f>
         <v>0</v>
       </c>
-      <c r="F18" s="79">
+      <c r="F18" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="88" t="s">
+      <c r="A19" s="86" t="s">
         <v>273</v>
       </c>
-      <c r="B19" s="38" t="s">
+      <c r="B19" s="36" t="s">
         <v>274</v>
       </c>
-      <c r="C19" s="78" t="s">
+      <c r="C19" s="76" t="s">
         <v>275</v>
       </c>
-      <c r="D19" s="78">
+      <c r="D19" s="76">
         <f>COUNTIF(Cronograma!$A$5:$A$37,$A19&amp;"*")</f>
         <v>4</v>
       </c>
-      <c r="E19" s="78">
+      <c r="E19" s="76">
         <f>COUNTIFS(Cronograma!$A$5:$A$37,$A19&amp;"*",Cronograma!$I$5:$I$37,"Hecho")</f>
         <v>0</v>
       </c>
-      <c r="F19" s="79">
+      <c r="F19" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="89" t="s">
+      <c r="A20" s="87" t="s">
         <v>276</v>
       </c>
-      <c r="B20" s="38" t="s">
+      <c r="B20" s="36" t="s">
         <v>277</v>
       </c>
-      <c r="C20" s="78" t="s">
+      <c r="C20" s="76" t="s">
         <v>278</v>
       </c>
-      <c r="D20" s="78">
+      <c r="D20" s="76">
         <f>COUNTIF(Cronograma!$A$5:$A$37,$A20&amp;"*")</f>
         <v>5</v>
       </c>
-      <c r="E20" s="78">
+      <c r="E20" s="76">
         <f>COUNTIFS(Cronograma!$A$5:$A$37,$A20&amp;"*",Cronograma!$I$5:$I$37,"Hecho")</f>
         <v>0</v>
       </c>
-      <c r="F20" s="79">
+      <c r="F20" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="90" t="s">
+      <c r="A21" s="88" t="s">
         <v>279</v>
       </c>
-      <c r="B21" s="39" t="s">
+      <c r="B21" s="37" t="s">
         <v>280</v>
       </c>
-      <c r="C21" s="80" t="s">
+      <c r="C21" s="78" t="s">
         <v>281</v>
       </c>
-      <c r="D21" s="80">
+      <c r="D21" s="78">
         <f>COUNTIF(Cronograma!$A$5:$A$37,$A21&amp;"*")</f>
         <v>3</v>
       </c>
-      <c r="E21" s="80">
+      <c r="E21" s="78">
         <f>COUNTIFS(Cronograma!$A$5:$A$37,$A21&amp;"*",Cronograma!$I$5:$I$37,"Hecho")</f>
         <v>0</v>
       </c>
-      <c r="F21" s="81">
+      <c r="F21" s="79">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="73" t="s">
+      <c r="A23" s="71" t="s">
         <v>282</v>
       </c>
       <c r="B23" s="4"/>
-      <c r="C23" s="71"/>
-      <c r="D23" s="82">
+      <c r="C23" s="69"/>
+      <c r="D23" s="80">
         <f>SUM(D14:D21)</f>
         <v>33</v>
       </c>
-      <c r="E23" s="82">
+      <c r="E23" s="80">
         <f>SUM(E14:E21)</f>
         <v>0</v>
       </c>
-      <c r="F23" s="72">
+      <c r="F23" s="70">
         <f>IF(D23=0,0,E23/D23)</f>
         <v>0</v>
       </c>
@@ -4595,43 +4943,731 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718FA6AC-696E-450F-994C-FF3B5BB5922F}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
+    <col min="2" max="2" width="49.5703125" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="28.5703125" customWidth="1"/>
+    <col min="7" max="7" width="57.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="94" t="s">
         <v>283</v>
       </c>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="32" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+    </row>
+    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="123" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="123" t="s">
         <v>285</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="124" t="s">
         <v>286</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="124" t="s">
         <v>287</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="124" t="s">
+        <v>291</v>
+      </c>
+      <c r="F4" s="124" t="s">
         <v>288</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="G4" s="124" t="s">
         <v>289</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>291</v>
-      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="104" t="s">
+        <v>292</v>
+      </c>
+      <c r="B5" s="98" t="s">
+        <v>293</v>
+      </c>
+      <c r="C5" s="110">
+        <v>1</v>
+      </c>
+      <c r="D5" s="111">
+        <v>60</v>
+      </c>
+      <c r="E5" s="107">
+        <f>C5*D5</f>
+        <v>60</v>
+      </c>
+      <c r="F5" s="95" t="s">
+        <v>325</v>
+      </c>
+      <c r="G5" s="101" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="105" t="s">
+        <v>292</v>
+      </c>
+      <c r="B6" s="99" t="s">
+        <v>294</v>
+      </c>
+      <c r="C6" s="112">
+        <v>1</v>
+      </c>
+      <c r="D6" s="113">
+        <v>200</v>
+      </c>
+      <c r="E6" s="108">
+        <f>C6*D6</f>
+        <v>200</v>
+      </c>
+      <c r="F6" s="96" t="s">
+        <v>327</v>
+      </c>
+      <c r="G6" s="102" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="105" t="s">
+        <v>292</v>
+      </c>
+      <c r="B7" s="99" t="s">
+        <v>295</v>
+      </c>
+      <c r="C7" s="112">
+        <v>1</v>
+      </c>
+      <c r="D7" s="113">
+        <v>12</v>
+      </c>
+      <c r="E7" s="108">
+        <f>C7*D7</f>
+        <v>12</v>
+      </c>
+      <c r="F7" s="96" t="s">
+        <v>329</v>
+      </c>
+      <c r="G7" s="102" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="105" t="s">
+        <v>292</v>
+      </c>
+      <c r="B8" s="99" t="s">
+        <v>296</v>
+      </c>
+      <c r="C8" s="112">
+        <v>1</v>
+      </c>
+      <c r="D8" s="113">
+        <v>10</v>
+      </c>
+      <c r="E8" s="108">
+        <f>C8*D8</f>
+        <v>10</v>
+      </c>
+      <c r="F8" s="96" t="s">
+        <v>331</v>
+      </c>
+      <c r="G8" s="102" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A9" s="105" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="99" t="s">
+        <v>297</v>
+      </c>
+      <c r="C9" s="112">
+        <v>6</v>
+      </c>
+      <c r="D9" s="113">
+        <v>200</v>
+      </c>
+      <c r="E9" s="108">
+        <f>C9*D9</f>
+        <v>1200</v>
+      </c>
+      <c r="F9" s="96" t="s">
+        <v>327</v>
+      </c>
+      <c r="G9" s="102" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="105" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="99" t="s">
+        <v>298</v>
+      </c>
+      <c r="C10" s="112">
+        <v>6</v>
+      </c>
+      <c r="D10" s="113">
+        <v>35</v>
+      </c>
+      <c r="E10" s="108">
+        <f>C10*D10</f>
+        <v>210</v>
+      </c>
+      <c r="F10" s="96" t="s">
+        <v>334</v>
+      </c>
+      <c r="G10" s="102" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A11" s="105" t="s">
+        <v>299</v>
+      </c>
+      <c r="B11" s="99" t="s">
+        <v>300</v>
+      </c>
+      <c r="C11" s="112">
+        <v>1</v>
+      </c>
+      <c r="D11" s="113">
+        <v>300</v>
+      </c>
+      <c r="E11" s="108">
+        <f>C11*D11</f>
+        <v>300</v>
+      </c>
+      <c r="F11" s="96" t="s">
+        <v>336</v>
+      </c>
+      <c r="G11" s="102" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="105" t="s">
+        <v>299</v>
+      </c>
+      <c r="B12" s="99" t="s">
+        <v>301</v>
+      </c>
+      <c r="C12" s="112">
+        <v>1</v>
+      </c>
+      <c r="D12" s="113">
+        <v>80</v>
+      </c>
+      <c r="E12" s="108">
+        <f>C12*D12</f>
+        <v>80</v>
+      </c>
+      <c r="F12" s="96" t="s">
+        <v>338</v>
+      </c>
+      <c r="G12" s="102" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="105" t="s">
+        <v>299</v>
+      </c>
+      <c r="B13" s="99" t="s">
+        <v>302</v>
+      </c>
+      <c r="C13" s="112">
+        <v>1</v>
+      </c>
+      <c r="D13" s="113">
+        <v>35</v>
+      </c>
+      <c r="E13" s="108">
+        <f>C13*D13</f>
+        <v>35</v>
+      </c>
+      <c r="F13" s="96" t="s">
+        <v>340</v>
+      </c>
+      <c r="G13" s="102" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="105" t="s">
+        <v>299</v>
+      </c>
+      <c r="B14" s="99" t="s">
+        <v>303</v>
+      </c>
+      <c r="C14" s="112">
+        <v>1</v>
+      </c>
+      <c r="D14" s="113">
+        <v>12</v>
+      </c>
+      <c r="E14" s="108">
+        <f>C14*D14</f>
+        <v>12</v>
+      </c>
+      <c r="F14" s="96" t="s">
+        <v>331</v>
+      </c>
+      <c r="G14" s="102" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="105" t="s">
+        <v>299</v>
+      </c>
+      <c r="B15" s="99" t="s">
+        <v>304</v>
+      </c>
+      <c r="C15" s="112">
+        <v>1</v>
+      </c>
+      <c r="D15" s="113">
+        <v>8</v>
+      </c>
+      <c r="E15" s="108">
+        <f>C15*D15</f>
+        <v>8</v>
+      </c>
+      <c r="F15" s="96" t="s">
+        <v>343</v>
+      </c>
+      <c r="G15" s="102" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="105" t="s">
+        <v>299</v>
+      </c>
+      <c r="B16" s="99" t="s">
+        <v>305</v>
+      </c>
+      <c r="C16" s="112">
+        <v>1</v>
+      </c>
+      <c r="D16" s="113">
+        <v>30</v>
+      </c>
+      <c r="E16" s="108">
+        <f>C16*D16</f>
+        <v>30</v>
+      </c>
+      <c r="F16" s="96" t="s">
+        <v>345</v>
+      </c>
+      <c r="G16" s="102" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="105" t="s">
+        <v>94</v>
+      </c>
+      <c r="B17" s="99" t="s">
+        <v>306</v>
+      </c>
+      <c r="C17" s="112">
+        <v>1</v>
+      </c>
+      <c r="D17" s="113">
+        <v>75</v>
+      </c>
+      <c r="E17" s="108">
+        <f>C17*D17</f>
+        <v>75</v>
+      </c>
+      <c r="F17" s="96" t="s">
+        <v>340</v>
+      </c>
+      <c r="G17" s="102" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="105" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="99" t="s">
+        <v>307</v>
+      </c>
+      <c r="C18" s="112">
+        <v>1</v>
+      </c>
+      <c r="D18" s="113">
+        <v>40</v>
+      </c>
+      <c r="E18" s="108">
+        <f>C18*D18</f>
+        <v>40</v>
+      </c>
+      <c r="F18" s="96" t="s">
+        <v>340</v>
+      </c>
+      <c r="G18" s="102" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="24" x14ac:dyDescent="0.25">
+      <c r="A19" s="105" t="s">
+        <v>308</v>
+      </c>
+      <c r="B19" s="99" t="s">
+        <v>309</v>
+      </c>
+      <c r="C19" s="112">
+        <v>2</v>
+      </c>
+      <c r="D19" s="113">
+        <v>130</v>
+      </c>
+      <c r="E19" s="108">
+        <f>C19*D19</f>
+        <v>260</v>
+      </c>
+      <c r="F19" s="96" t="s">
+        <v>340</v>
+      </c>
+      <c r="G19" s="102" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="105" t="s">
+        <v>308</v>
+      </c>
+      <c r="B20" s="99" t="s">
+        <v>310</v>
+      </c>
+      <c r="C20" s="112">
+        <v>1</v>
+      </c>
+      <c r="D20" s="113">
+        <v>400</v>
+      </c>
+      <c r="E20" s="108">
+        <f>C20*D20</f>
+        <v>400</v>
+      </c>
+      <c r="F20" s="96" t="s">
+        <v>340</v>
+      </c>
+      <c r="G20" s="102" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="105" t="s">
+        <v>308</v>
+      </c>
+      <c r="B21" s="99" t="s">
+        <v>311</v>
+      </c>
+      <c r="C21" s="112">
+        <v>1</v>
+      </c>
+      <c r="D21" s="113">
+        <v>15</v>
+      </c>
+      <c r="E21" s="108">
+        <f>C21*D21</f>
+        <v>15</v>
+      </c>
+      <c r="F21" s="96" t="s">
+        <v>343</v>
+      </c>
+      <c r="G21" s="102" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="105" t="s">
+        <v>308</v>
+      </c>
+      <c r="B22" s="99" t="s">
+        <v>312</v>
+      </c>
+      <c r="C22" s="112">
+        <v>1</v>
+      </c>
+      <c r="D22" s="113">
+        <v>25</v>
+      </c>
+      <c r="E22" s="108">
+        <f>C22*D22</f>
+        <v>25</v>
+      </c>
+      <c r="F22" s="96" t="s">
+        <v>331</v>
+      </c>
+      <c r="G22" s="102" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="105" t="s">
+        <v>313</v>
+      </c>
+      <c r="B23" s="99" t="s">
+        <v>314</v>
+      </c>
+      <c r="C23" s="112">
+        <v>1</v>
+      </c>
+      <c r="D23" s="113">
+        <v>100</v>
+      </c>
+      <c r="E23" s="108">
+        <f>C23*D23</f>
+        <v>100</v>
+      </c>
+      <c r="F23" s="96" t="s">
+        <v>334</v>
+      </c>
+      <c r="G23" s="102" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="105" t="s">
+        <v>313</v>
+      </c>
+      <c r="B24" s="99" t="s">
+        <v>315</v>
+      </c>
+      <c r="C24" s="112">
+        <v>2</v>
+      </c>
+      <c r="D24" s="113">
+        <v>90</v>
+      </c>
+      <c r="E24" s="108">
+        <f>C24*D24</f>
+        <v>180</v>
+      </c>
+      <c r="F24" s="96" t="s">
+        <v>334</v>
+      </c>
+      <c r="G24" s="102" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="105" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="99" t="s">
+        <v>316</v>
+      </c>
+      <c r="C25" s="112">
+        <v>1</v>
+      </c>
+      <c r="D25" s="113">
+        <v>250</v>
+      </c>
+      <c r="E25" s="108">
+        <f>C25*D25</f>
+        <v>250</v>
+      </c>
+      <c r="F25" s="96" t="s">
+        <v>340</v>
+      </c>
+      <c r="G25" s="102" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="105" t="s">
+        <v>122</v>
+      </c>
+      <c r="B26" s="99" t="s">
+        <v>317</v>
+      </c>
+      <c r="C26" s="112">
+        <v>1</v>
+      </c>
+      <c r="D26" s="113">
+        <v>60</v>
+      </c>
+      <c r="E26" s="108">
+        <f>C26*D26</f>
+        <v>60</v>
+      </c>
+      <c r="F26" s="96" t="s">
+        <v>340</v>
+      </c>
+      <c r="G26" s="102" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="105" t="s">
+        <v>122</v>
+      </c>
+      <c r="B27" s="99" t="s">
+        <v>318</v>
+      </c>
+      <c r="C27" s="112">
+        <v>1</v>
+      </c>
+      <c r="D27" s="113">
+        <v>25</v>
+      </c>
+      <c r="E27" s="108">
+        <f>C27*D27</f>
+        <v>25</v>
+      </c>
+      <c r="F27" s="96" t="s">
+        <v>340</v>
+      </c>
+      <c r="G27" s="102" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="105" t="s">
+        <v>122</v>
+      </c>
+      <c r="B28" s="99" t="s">
+        <v>319</v>
+      </c>
+      <c r="C28" s="112">
+        <v>1</v>
+      </c>
+      <c r="D28" s="113">
+        <v>150</v>
+      </c>
+      <c r="E28" s="108">
+        <f>C28*D28</f>
+        <v>150</v>
+      </c>
+      <c r="F28" s="96" t="s">
+        <v>358</v>
+      </c>
+      <c r="G28" s="102" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="105" t="s">
+        <v>122</v>
+      </c>
+      <c r="B29" s="99" t="s">
+        <v>320</v>
+      </c>
+      <c r="C29" s="112">
+        <v>1</v>
+      </c>
+      <c r="D29" s="113">
+        <v>60</v>
+      </c>
+      <c r="E29" s="108">
+        <f>C29*D29</f>
+        <v>60</v>
+      </c>
+      <c r="F29" s="96" t="s">
+        <v>343</v>
+      </c>
+      <c r="G29" s="102" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="105" t="s">
+        <v>321</v>
+      </c>
+      <c r="B30" s="99" t="s">
+        <v>322</v>
+      </c>
+      <c r="C30" s="112">
+        <v>1</v>
+      </c>
+      <c r="D30" s="113">
+        <v>40</v>
+      </c>
+      <c r="E30" s="108">
+        <f>C30*D30</f>
+        <v>40</v>
+      </c>
+      <c r="F30" s="96" t="s">
+        <v>343</v>
+      </c>
+      <c r="G30" s="102" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="106" t="s">
+        <v>323</v>
+      </c>
+      <c r="B31" s="100" t="s">
+        <v>324</v>
+      </c>
+      <c r="C31" s="114">
+        <v>1</v>
+      </c>
+      <c r="D31" s="115">
+        <v>40</v>
+      </c>
+      <c r="E31" s="109">
+        <f>C31*D31</f>
+        <v>40</v>
+      </c>
+      <c r="F31" s="97" t="s">
+        <v>343</v>
+      </c>
+      <c r="G31" s="103" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="120" t="s">
+        <v>363</v>
+      </c>
+      <c r="B32" s="116"/>
+      <c r="C32" s="116"/>
+      <c r="D32" s="117"/>
+      <c r="E32" s="118">
+        <f>SUM(E5:E31)</f>
+        <v>3877</v>
+      </c>
+      <c r="F32" s="119"/>
+      <c r="G32" s="119"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4648,144 +5684,144 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="31" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="32" t="s">
         <v>177</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="33" t="s">
         <v>178</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="34" t="s">
         <v>180</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="35" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="40" t="s">
+      <c r="A5" s="38" t="s">
         <v>181</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="40" t="s">
         <v>182</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="42" t="s">
         <v>183</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="44" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="B6" s="42" t="s">
+      <c r="B6" s="40" t="s">
         <v>184</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="42" t="s">
         <v>185</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="44" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="B7" s="42" t="s">
+      <c r="B7" s="40" t="s">
         <v>186</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="42" t="s">
         <v>187</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="44" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="40" t="s">
         <v>188</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="44" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="38" t="s">
         <v>151</v>
       </c>
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="40" t="s">
         <v>190</v>
       </c>
-      <c r="C9" s="44" t="s">
+      <c r="C9" s="42" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D9" s="44" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="40" t="s">
+      <c r="A10" s="38" t="s">
         <v>155</v>
       </c>
-      <c r="B10" s="42" t="s">
+      <c r="B10" s="40" t="s">
         <v>192</v>
       </c>
-      <c r="C10" s="44" t="s">
+      <c r="C10" s="42" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="46" t="s">
+      <c r="D10" s="44" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="40" t="s">
+      <c r="A11" s="38" t="s">
         <v>164</v>
       </c>
-      <c r="B11" s="42" t="s">
+      <c r="B11" s="40" t="s">
         <v>194</v>
       </c>
-      <c r="C11" s="44" t="s">
+      <c r="C11" s="42" t="s">
         <v>195</v>
       </c>
-      <c r="D11" s="46" t="s">
+      <c r="D11" s="44" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="41" t="s">
         <v>197</v>
       </c>
-      <c r="C12" s="45" t="s">
+      <c r="C12" s="43" t="s">
         <v>198</v>
       </c>
-      <c r="D12" s="47" t="s">
+      <c r="D12" s="45" t="s">
         <v>21</v>
       </c>
     </row>
@@ -4835,130 +5871,130 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="46" t="s">
         <v>199</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="47" t="s">
         <v>200</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="48" t="s">
         <v>201</v>
       </c>
-      <c r="B4" s="51" t="s">
+      <c r="B4" s="49" t="s">
         <v>202</v>
       </c>
-      <c r="C4" s="51" t="s">
+      <c r="C4" s="49" t="s">
         <v>203</v>
       </c>
-      <c r="D4" s="52" t="s">
+      <c r="D4" s="50" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="55" t="s">
+      <c r="A5" s="53" t="s">
         <v>205</v>
       </c>
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="51" t="s">
         <v>206</v>
       </c>
-      <c r="C5" s="53" t="s">
+      <c r="C5" s="51" t="s">
         <v>207</v>
       </c>
-      <c r="D5" s="57" t="s">
+      <c r="D5" s="55" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="55" t="s">
+      <c r="A6" s="53" t="s">
         <v>209</v>
       </c>
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="51" t="s">
         <v>206</v>
       </c>
-      <c r="C6" s="53" t="s">
+      <c r="C6" s="51" t="s">
         <v>207</v>
       </c>
-      <c r="D6" s="57" t="s">
+      <c r="D6" s="55" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="53" t="s">
         <v>211</v>
       </c>
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="51" t="s">
         <v>212</v>
       </c>
-      <c r="C7" s="53" t="s">
+      <c r="C7" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="D7" s="57" t="s">
+      <c r="D7" s="55" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="55" t="s">
+      <c r="A8" s="53" t="s">
         <v>215</v>
       </c>
-      <c r="B8" s="53">
+      <c r="B8" s="51">
         <v>3</v>
       </c>
-      <c r="C8" s="53" t="s">
+      <c r="C8" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="D8" s="57" t="s">
+      <c r="D8" s="55" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="55" t="s">
+      <c r="A9" s="53" t="s">
         <v>217</v>
       </c>
-      <c r="B9" s="53">
+      <c r="B9" s="51">
         <v>8</v>
       </c>
-      <c r="C9" s="53" t="s">
+      <c r="C9" s="51" t="s">
         <v>207</v>
       </c>
-      <c r="D9" s="57" t="s">
+      <c r="D9" s="55" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="55" t="s">
+      <c r="A10" s="53" t="s">
         <v>219</v>
       </c>
-      <c r="B10" s="53" t="s">
+      <c r="B10" s="51" t="s">
         <v>206</v>
       </c>
-      <c r="C10" s="53" t="s">
+      <c r="C10" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="D10" s="57" t="s">
+      <c r="D10" s="55" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="56" t="s">
+      <c r="A11" s="54" t="s">
         <v>221</v>
       </c>
-      <c r="B11" s="54" t="s">
+      <c r="B11" s="52" t="s">
         <v>222</v>
       </c>
-      <c r="C11" s="54" t="s">
+      <c r="C11" s="52" t="s">
         <v>213</v>
       </c>
-      <c r="D11" s="58" t="s">
+      <c r="D11" s="56" t="s">
         <v>223</v>
       </c>
     </row>
@@ -4991,107 +6027,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="58" t="s">
         <v>224</v>
       </c>
-      <c r="B1" s="60"/>
+      <c r="B1" s="58"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="59" t="s">
         <v>225</v>
       </c>
-      <c r="B2" s="61"/>
+      <c r="B2" s="59"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="62" t="s">
+      <c r="A4" s="60" t="s">
         <v>226</v>
       </c>
-      <c r="B4" s="63" t="s">
+      <c r="B4" s="61" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="64">
+      <c r="A5" s="62">
         <v>1</v>
       </c>
-      <c r="B5" s="66" t="s">
+      <c r="B5" s="64" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="64">
+      <c r="A6" s="62">
         <v>2</v>
       </c>
-      <c r="B6" s="66" t="s">
+      <c r="B6" s="64" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="64">
+      <c r="A7" s="62">
         <v>3</v>
       </c>
-      <c r="B7" s="66" t="s">
+      <c r="B7" s="64" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="64">
+      <c r="A8" s="62">
         <v>4</v>
       </c>
-      <c r="B8" s="66" t="s">
+      <c r="B8" s="64" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="65">
+      <c r="A9" s="63">
         <v>5</v>
       </c>
-      <c r="B9" s="67" t="s">
+      <c r="B9" s="65" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="59" t="s">
+      <c r="A11" s="57" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="68" t="s">
+      <c r="A12" s="66" t="s">
         <v>234</v>
       </c>
-      <c r="B12" s="69" t="s">
+      <c r="B12" s="67" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="68" t="s">
+      <c r="A13" s="66" t="s">
         <v>234</v>
       </c>
-      <c r="B13" s="69" t="s">
+      <c r="B13" s="67" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="68" t="s">
+      <c r="A14" s="66" t="s">
         <v>234</v>
       </c>
-      <c r="B14" s="69" t="s">
+      <c r="B14" s="67" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="68" t="s">
+      <c r="A15" s="66" t="s">
         <v>234</v>
       </c>
-      <c r="B15" s="69" t="s">
+      <c r="B15" s="67" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="68" t="s">
+      <c r="A16" s="66" t="s">
         <v>234</v>
       </c>
-      <c r="B16" s="69" t="s">
+      <c r="B16" s="67" t="s">
         <v>239</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualizar docs + nuevo analisis MAVLink/BlueOS
</commit_message>
<xml_diff>
--- a/Plan_cosntruccion.xlsx
+++ b/Plan_cosntruccion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Rov\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F94433-34B5-48A3-B175-231797A0AA24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4932424A-4B2C-447B-A7C4-1FF71679D538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{75C40051-293E-4382-8A6D-0D6B95F2BCBB}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="1" activeTab="1" xr2:uid="{75C40051-293E-4382-8A6D-0D6B95F2BCBB}"/>
   </bookViews>
   <sheets>
     <sheet name="Tablero" sheetId="2" r:id="rId1"/>

</xml_diff>